<commit_message>
docs: update Db.xlsx, UC diagram and ignore Draw.io backup files
</commit_message>
<xml_diff>
--- a/docs/Database/Db.xlsx
+++ b/docs/Database/Db.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Đặt lịch phòng khám\docs\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Đặt lịch phòng khám\Đặt lịch phòng khám BA\docs\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CD8855-8CA7-4BF9-8497-FA40AA194662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30320DD9-DC58-484E-9922-04067CD6D7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="97">
   <si>
     <t>Users</t>
   </si>
@@ -219,12 +219,105 @@
   <si>
     <t>author_id</t>
   </si>
+  <si>
+    <t>Medical_Records</t>
+  </si>
+  <si>
+    <t>appointment_id</t>
+  </si>
+  <si>
+    <t>record_code</t>
+  </si>
+  <si>
+    <t>clinical_examination</t>
+  </si>
+  <si>
+    <t>diagnosis</t>
+  </si>
+  <si>
+    <t>icd10_code</t>
+  </si>
+  <si>
+    <t>icd10_name</t>
+  </si>
+  <si>
+    <t>blood_pressure</t>
+  </si>
+  <si>
+    <t>pulse</t>
+  </si>
+  <si>
+    <t>temperature</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>doctor_advice</t>
+  </si>
+  <si>
+    <t>re_examination_date</t>
+  </si>
+  <si>
+    <t>consultation_type</t>
+  </si>
+  <si>
+    <t>recommendation</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>Medical_Records_Attachments</t>
+  </si>
+  <si>
+    <t>medical_record_id</t>
+  </si>
+  <si>
+    <t>file_url</t>
+  </si>
+  <si>
+    <t>file_name</t>
+  </si>
+  <si>
+    <t>Prescription_Items</t>
+  </si>
+  <si>
+    <t>medicine_name</t>
+  </si>
+  <si>
+    <t>dosage</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>instructions</t>
+  </si>
+  <si>
+    <t>Nhóm Hồ sơ bệnh án (Mối quan hệ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MedicalRecord </t>
+  </si>
+  <si>
+    <t>PrescriptionItem</t>
+  </si>
+  <si>
+    <t>MedicalRecordAttachment</t>
+  </si>
+  <si>
+    <t>signed_at</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,8 +384,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF555555"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -394,8 +535,24 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -577,54 +734,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -637,80 +769,40 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -739,9 +831,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -774,53 +863,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="14" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="15" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -829,9 +873,78 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="4" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="4" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="6">
+    <cellStyle name="20% - Accent1" xfId="4" builtinId="30"/>
     <cellStyle name="60% - Accent5" xfId="2" builtinId="48"/>
+    <cellStyle name="Accent1" xfId="3" builtinId="29"/>
+    <cellStyle name="Accent2" xfId="5" builtinId="33"/>
     <cellStyle name="Accent5" xfId="1" builtinId="45"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1176,29 +1289,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="21"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="21"/>
+      <c r="Q1" s="11"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -1210,29 +1316,33 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="26" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="43" t="s">
+      <c r="E2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="11"/>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
@@ -1244,29 +1354,33 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="26" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="43" t="s">
+      <c r="E3" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="11"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -1278,29 +1392,33 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="26" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="12"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="N4" s="37"/>
+      <c r="O4" s="37"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="11"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
@@ -1312,29 +1430,33 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="26" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="11"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
@@ -1346,29 +1468,33 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="26" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>55</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="44" t="s">
+      <c r="E6" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="11"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
@@ -1380,27 +1506,31 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="26" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="37"/>
+      <c r="O7" s="37"/>
+      <c r="P7" s="37"/>
+      <c r="Q7" s="11"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
@@ -1412,26 +1542,30 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="26" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="29" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="N8" s="37"/>
+      <c r="O8" s="37"/>
+      <c r="P8" s="37"/>
+      <c r="Q8" s="11"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
@@ -1443,26 +1577,28 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="27" t="s">
         <v>55</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="26" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -1475,23 +1611,27 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="26" t="s">
         <v>64</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="3"/>
-      <c r="K10" s="1"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="11"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -1505,22 +1645,24 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="26" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="2"/>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="26" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="42" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" s="42"/>
+      <c r="J11" s="42"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="21"/>
+      <c r="P11" s="11"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
@@ -1534,21 +1676,28 @@
     </row>
     <row r="12" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="2"/>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="26" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="N12" s="40"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="11"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -1562,21 +1711,28 @@
     </row>
     <row r="13" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B13" s="2"/>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="26" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="N13" s="37"/>
+      <c r="O13" s="37"/>
+      <c r="P13" s="11"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -1589,25 +1745,32 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="2"/>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="26" t="s">
         <v>28</v>
       </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="N14" s="37"/>
+      <c r="O14" s="37"/>
+      <c r="P14" s="11"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -1620,25 +1783,32 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2"/>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="26" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="2"/>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="N15" s="37"/>
+      <c r="O15" s="37"/>
+      <c r="P15" s="11"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -1651,25 +1821,32 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="26" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="2"/>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="12"/>
-      <c r="G16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="N16" s="37"/>
+      <c r="O16" s="37"/>
+      <c r="P16" s="32"/>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -1682,26 +1859,33 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="2"/>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="26" t="s">
         <v>32</v>
       </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="42" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="N17" s="37"/>
+      <c r="O17" s="37"/>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="11"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
@@ -1713,25 +1897,32 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="2"/>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="26" t="s">
         <v>34</v>
       </c>
       <c r="D18" s="2"/>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="N18" s="37"/>
+      <c r="O18" s="37"/>
+      <c r="P18" s="33"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -1744,25 +1935,32 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>25</v>
       </c>
       <c r="B19" s="2"/>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="26" t="s">
         <v>35</v>
       </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="N19" s="37"/>
+      <c r="O19" s="37"/>
+      <c r="P19" s="11"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -1775,57 +1973,84 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B20" s="2"/>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="26" t="s">
         <v>36</v>
       </c>
       <c r="D20" s="2"/>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F20" s="14"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="42" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="13"/>
     </row>
     <row r="21" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="27" t="s">
         <v>55</v>
       </c>
       <c r="D21" s="2"/>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="13"/>
     </row>
     <row r="22" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
+      <c r="C22" s="26" t="s">
+        <v>62</v>
+      </c>
       <c r="D22" s="2"/>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="10" t="s">
         <v>55</v>
       </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="13"/>
     </row>
     <row r="23" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="15" t="s">
         <v>38</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="1"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="24"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
       <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="22"/>
+      <c r="Q23" s="22"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
@@ -1837,34 +2062,23 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="20" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="2"/>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D24" s="2"/>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="26"/>
-      <c r="G24" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="H24" s="39"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="L24" s="36"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="12"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
+      <c r="F24" s="24"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="48"/>
+      <c r="N24" s="24"/>
+      <c r="R24" s="11"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
@@ -1875,34 +2089,21 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B25" s="2"/>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D25" s="2"/>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F25" s="26"/>
-      <c r="G25" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="28"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="12"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
+      <c r="F25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="R25" s="11"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
@@ -1913,34 +2114,21 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B26" s="2"/>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="2"/>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="26"/>
-      <c r="G26" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="H26" s="28"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="L26" s="28"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
+      <c r="F26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="R26" s="11"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
@@ -1951,34 +2139,21 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="17" t="s">
         <v>41</v>
       </c>
       <c r="B27" s="2"/>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="F27" s="26"/>
-      <c r="G27" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" s="28"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="L27" s="28"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1"/>
-      <c r="R27" s="1"/>
+      <c r="F27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="R27" s="11"/>
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
@@ -1991,28 +2166,15 @@
     <row r="28" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="L28" s="28"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="12"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="1"/>
-      <c r="R28" s="1"/>
+      <c r="F28" s="21"/>
+      <c r="J28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="R28" s="11"/>
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
@@ -2025,28 +2187,20 @@
     <row r="29" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="30" t="s">
-        <v>14</v>
+      <c r="F29" s="21"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="50" t="s">
+        <v>56</v>
       </c>
-      <c r="H29" s="31"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L29" s="28"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="12"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="50"/>
+      <c r="N29" s="24"/>
+      <c r="R29" s="11"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
@@ -2059,28 +2213,27 @@
     <row r="30" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>55</v>
       </c>
       <c r="D30" s="2"/>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="27" t="s">
-        <v>60</v>
+      <c r="F30" s="24"/>
+      <c r="G30" s="49" t="s">
+        <v>61</v>
       </c>
-      <c r="L30" s="28"/>
-      <c r="M30" s="29"/>
-      <c r="N30" s="12"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="L30" s="37"/>
+      <c r="M30" s="37"/>
+      <c r="N30" s="24"/>
+      <c r="R30" s="11"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
@@ -2094,24 +2247,23 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="27" t="s">
-        <v>33</v>
+      <c r="F31" s="24"/>
+      <c r="G31" s="37" t="s">
+        <v>3</v>
       </c>
-      <c r="L31" s="28"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="12"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="L31" s="37"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="24"/>
+      <c r="R31" s="11"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
@@ -2122,32 +2274,31 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="19" t="s">
         <v>43</v>
       </c>
       <c r="B32" s="2"/>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="19" t="s">
         <v>44</v>
       </c>
       <c r="D32" s="2"/>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="30" t="s">
-        <v>55</v>
+      <c r="F32" s="24"/>
+      <c r="G32" s="37" t="s">
+        <v>62</v>
       </c>
-      <c r="L32" s="31"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="12"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
-      <c r="R32" s="1"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="L32" s="37"/>
+      <c r="M32" s="37"/>
+      <c r="N32" s="24"/>
+      <c r="R32" s="11"/>
       <c r="S32" s="1"/>
       <c r="T32" s="1"/>
       <c r="U32" s="1"/>
@@ -2158,30 +2309,34 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D33" s="2"/>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F33" s="12"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="L33" s="37"/>
+      <c r="M33" s="37"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="11"/>
       <c r="S33" s="1"/>
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
@@ -2192,30 +2347,34 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B34" s="2"/>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D34" s="2"/>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F34" s="12"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="L34" s="37"/>
+      <c r="M34" s="37"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="46"/>
+      <c r="Q34" s="46"/>
+      <c r="R34" s="11"/>
       <c r="S34" s="1"/>
       <c r="T34" s="1"/>
       <c r="U34" s="1"/>
@@ -2226,30 +2385,34 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="17" t="s">
         <v>36</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="2"/>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-      <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-      <c r="P35" s="1"/>
-      <c r="Q35" s="1"/>
-      <c r="R35" s="1"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="L35" s="37"/>
+      <c r="M35" s="37"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="46"/>
+      <c r="Q35" s="46"/>
+      <c r="R35" s="11"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
@@ -2262,26 +2425,28 @@
     <row r="36" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>47</v>
       </c>
       <c r="D36" s="2"/>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F36" s="12"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
-      <c r="Q36" s="1"/>
-      <c r="R36" s="1"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="24"/>
+      <c r="K36" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="L36" s="37"/>
+      <c r="M36" s="37"/>
+      <c r="N36" s="24"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="46"/>
+      <c r="Q36" s="46"/>
+      <c r="R36" s="11"/>
       <c r="S36" s="1"/>
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
@@ -2294,22 +2459,24 @@
     <row r="37" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="19" t="s">
+      <c r="C37" s="17" t="s">
         <v>14</v>
       </c>
       <c r="D37" s="2"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
-      <c r="Q37" s="1"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="L37" s="37"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="23"/>
+      <c r="Q37" s="23"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
@@ -2329,11 +2496,11 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="11"/>
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
@@ -2348,22 +2515,22 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="26.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="33" t="s">
+      <c r="A39" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
-      <c r="K39" s="1"/>
-      <c r="L39" s="1"/>
-      <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="46"/>
+      <c r="M39" s="46"/>
+      <c r="N39" s="11"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
@@ -2378,13 +2545,13 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="4">
+      <c r="A40" s="3">
         <v>1</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D40" s="2"/>
@@ -2393,11 +2560,11 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="46"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="46"/>
+      <c r="N40" s="11"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
@@ -2412,13 +2579,13 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D41" s="2"/>
@@ -2428,9 +2595,9 @@
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
@@ -2474,13 +2641,13 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A43" s="4">
+      <c r="A43" s="3">
         <v>1</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D43" s="2"/>
@@ -2508,13 +2675,13 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D44" s="2"/>
@@ -2570,13 +2737,13 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A46" s="4">
+      <c r="A46" s="3">
         <v>1</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D46" s="2"/>
@@ -2604,13 +2771,13 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D47" s="2"/>
@@ -2666,13 +2833,13 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A49" s="4">
+      <c r="A49" s="3">
         <v>1</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D49" s="2"/>
@@ -2700,13 +2867,13 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="B50" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D50" s="2"/>
@@ -2762,13 +2929,13 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A52" s="4">
+      <c r="A52" s="3">
         <v>1</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D52" s="2"/>
@@ -2796,13 +2963,13 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B53" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D53" s="2"/>
@@ -2858,13 +3025,13 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A55" s="4">
+      <c r="A55" s="3">
         <v>1</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D55" s="2"/>
@@ -2892,13 +3059,13 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B56" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D56" s="2"/>
@@ -2954,13 +3121,13 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="4">
+      <c r="A58" s="3">
         <v>1</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C58" s="4">
+      <c r="C58" s="3">
         <v>1</v>
       </c>
       <c r="D58" s="2"/>
@@ -2988,13 +3155,13 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D59" s="2"/>
@@ -3022,26 +3189,26 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A60" s="4">
+      <c r="A60" s="3">
         <v>1</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
     </row>
     <row r="61" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A61" s="6" t="s">
+      <c r="A61" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D61" s="2"/>
@@ -3083,13 +3250,13 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="26.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B64" s="34"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="34"/>
+      <c r="B64" s="39"/>
+      <c r="C64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="39"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
@@ -3113,13 +3280,13 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A65" s="4">
+      <c r="A65" s="3">
         <v>1</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C65" s="4">
+      <c r="C65" s="3">
         <v>1</v>
       </c>
       <c r="D65" s="2"/>
@@ -3147,13 +3314,13 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="B66" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D66" s="2"/>
@@ -3209,13 +3376,13 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A68" s="4">
+      <c r="A68" s="3">
         <v>1</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D68" s="2"/>
@@ -3243,13 +3410,13 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A69" s="6" t="s">
+      <c r="A69" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B69" s="7" t="s">
+      <c r="B69" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D69" s="2"/>
@@ -3305,13 +3472,13 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A71" s="4">
+      <c r="A71" s="3">
         <v>1</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="C71" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D71" s="2"/>
@@ -3339,13 +3506,13 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="6" t="s">
+      <c r="A72" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B72" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C72" s="6" t="s">
+      <c r="C72" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D72" s="2"/>
@@ -3401,13 +3568,13 @@
       <c r="Z73" s="1"/>
     </row>
     <row r="74" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A74" s="4">
+      <c r="A74" s="3">
         <v>1</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C74" s="4">
+      <c r="C74" s="3">
         <v>1</v>
       </c>
       <c r="D74" s="2"/>
@@ -3435,13 +3602,13 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A75" s="6" t="s">
+      <c r="A75" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="B75" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D75" s="2"/>
@@ -3497,13 +3664,13 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="33" t="s">
+      <c r="A77" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B77" s="34"/>
-      <c r="C77" s="34"/>
-      <c r="D77" s="34"/>
-      <c r="E77" s="34"/>
+      <c r="B77" s="39"/>
+      <c r="C77" s="39"/>
+      <c r="D77" s="39"/>
+      <c r="E77" s="39"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
@@ -3527,13 +3694,13 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A78" s="4">
+      <c r="A78" s="3">
         <v>1</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D78" s="2"/>
@@ -3561,13 +3728,13 @@
       <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A79" s="6" t="s">
+      <c r="A79" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B79" s="7" t="s">
+      <c r="B79" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C79" s="6" t="s">
+      <c r="C79" s="5" t="s">
         <v>63</v>
       </c>
       <c r="D79" s="2"/>
@@ -3623,13 +3790,13 @@
       <c r="Z80" s="1"/>
     </row>
     <row r="81" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A81" s="4">
+      <c r="A81" s="3">
         <v>1</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D81" s="2"/>
@@ -3657,13 +3824,13 @@
       <c r="Z81" s="1"/>
     </row>
     <row r="82" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A82" s="6" t="s">
+      <c r="A82" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B82" s="7" t="s">
+      <c r="B82" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C82" s="6" t="s">
+      <c r="C82" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D82" s="2"/>
@@ -3719,13 +3886,13 @@
       <c r="Z83" s="1"/>
     </row>
     <row r="84" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A84" s="4">
+      <c r="A84" s="3">
         <v>1</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D84" s="2"/>
@@ -3753,13 +3920,13 @@
       <c r="Z84" s="1"/>
     </row>
     <row r="85" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A85" s="6" t="s">
+      <c r="A85" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="7" t="s">
+      <c r="B85" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C85" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D85" s="2"/>
@@ -3815,14 +3982,14 @@
       <c r="Z86" s="1"/>
     </row>
     <row r="87" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A87" s="4">
+      <c r="A87" s="3">
         <v>1</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C87" s="4">
-        <v>1</v>
+      <c r="C87" s="35" t="s">
+        <v>53</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
@@ -3849,13 +4016,13 @@
       <c r="Z87" s="1"/>
     </row>
     <row r="88" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A88" s="6" t="s">
+      <c r="A88" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B88" s="7" t="s">
+      <c r="B88" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D88" s="2"/>
@@ -3910,12 +4077,14 @@
       <c r="Y89" s="1"/>
       <c r="Z89" s="1"/>
     </row>
-    <row r="90" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
+    <row r="90" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A90" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="39"/>
+      <c r="C90" s="39"/>
+      <c r="D90" s="39"/>
+      <c r="E90" s="39"/>
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
       <c r="H90" s="1"/>
@@ -3939,9 +4108,15 @@
       <c r="Z90" s="1"/>
     </row>
     <row r="91" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
+      <c r="A91" s="3">
+        <v>1</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C91" s="3">
+        <v>1</v>
+      </c>
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
       <c r="F91" s="1"/>
@@ -3967,9 +4142,15 @@
       <c r="Z91" s="1"/>
     </row>
     <row r="92" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="2"/>
+      <c r="A92" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C92" s="36" t="s">
+        <v>17</v>
+      </c>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
       <c r="F92" s="1"/>
@@ -4023,9 +4204,15 @@
       <c r="Z93" s="1"/>
     </row>
     <row r="94" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2"/>
+      <c r="A94" s="3">
+        <v>1</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
       <c r="F94" s="1"/>
@@ -4051,9 +4238,15 @@
       <c r="Z94" s="1"/>
     </row>
     <row r="95" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A95" s="2"/>
-      <c r="B95" s="2"/>
-      <c r="C95" s="2"/>
+      <c r="A95" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C95" s="36" t="s">
+        <v>94</v>
+      </c>
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
       <c r="F95" s="1"/>
@@ -4107,9 +4300,15 @@
       <c r="Z96" s="1"/>
     </row>
     <row r="97" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
+      <c r="A97" s="3">
+        <v>1</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
       <c r="F97" s="1"/>
@@ -4135,9 +4334,15 @@
       <c r="Z97" s="1"/>
     </row>
     <row r="98" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="2"/>
+      <c r="A98" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C98" s="36" t="s">
+        <v>95</v>
+      </c>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
       <c r="F98" s="1"/>
@@ -4190,12 +4395,12 @@
       <c r="Y99" s="1"/>
       <c r="Z99" s="1"/>
     </row>
-    <row r="100" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A100" s="1"/>
-      <c r="B100" s="1"/>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1"/>
-      <c r="E100" s="1"/>
+    <row r="100" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A100" s="3"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="35"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
@@ -4218,12 +4423,12 @@
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
     </row>
-    <row r="101" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A101" s="1"/>
-      <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
-      <c r="E101" s="1"/>
+    <row r="101" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A101" s="5"/>
+      <c r="B101" s="6"/>
+      <c r="C101" s="36"/>
+      <c r="D101" s="2"/>
+      <c r="E101" s="2"/>
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
@@ -29587,25 +29792,63 @@
       <c r="Z1006" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="56">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A64:E64"/>
     <mergeCell ref="A77:E77"/>
-    <mergeCell ref="K24:M24"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="K28:M28"/>
     <mergeCell ref="K29:M29"/>
     <mergeCell ref="K30:M30"/>
     <mergeCell ref="K31:M31"/>
     <mergeCell ref="K32:M32"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="M4:P4"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="M7:P7"/>
+    <mergeCell ref="M6:P6"/>
+    <mergeCell ref="M5:P5"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="M8:P8"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="H8:J8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Update(UC & Db) (#6)
* Design(UML):CREATE management Post and management Booking (Online and offline)

* docs: add sequence diagrams for doctor and specialty management modules

* chore: add .gitignore and untrack Visual Paradigm backup and temporary files

* docs: update Db.xlsx, UC diagram and ignore Draw.io backup files
</commit_message>
<xml_diff>
--- a/docs/Database/Db.xlsx
+++ b/docs/Database/Db.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Đặt lịch phòng khám\docs\Database\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Đặt lịch phòng khám\Đặt lịch phòng khám BA\docs\Database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80CD8855-8CA7-4BF9-8497-FA40AA194662}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30320DD9-DC58-484E-9922-04067CD6D7C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="97">
   <si>
     <t>Users</t>
   </si>
@@ -219,12 +219,105 @@
   <si>
     <t>author_id</t>
   </si>
+  <si>
+    <t>Medical_Records</t>
+  </si>
+  <si>
+    <t>appointment_id</t>
+  </si>
+  <si>
+    <t>record_code</t>
+  </si>
+  <si>
+    <t>clinical_examination</t>
+  </si>
+  <si>
+    <t>diagnosis</t>
+  </si>
+  <si>
+    <t>icd10_code</t>
+  </si>
+  <si>
+    <t>icd10_name</t>
+  </si>
+  <si>
+    <t>blood_pressure</t>
+  </si>
+  <si>
+    <t>pulse</t>
+  </si>
+  <si>
+    <t>temperature</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>doctor_advice</t>
+  </si>
+  <si>
+    <t>re_examination_date</t>
+  </si>
+  <si>
+    <t>consultation_type</t>
+  </si>
+  <si>
+    <t>recommendation</t>
+  </si>
+  <si>
+    <t>updated_at</t>
+  </si>
+  <si>
+    <t>Medical_Records_Attachments</t>
+  </si>
+  <si>
+    <t>medical_record_id</t>
+  </si>
+  <si>
+    <t>file_url</t>
+  </si>
+  <si>
+    <t>file_name</t>
+  </si>
+  <si>
+    <t>Prescription_Items</t>
+  </si>
+  <si>
+    <t>medicine_name</t>
+  </si>
+  <si>
+    <t>dosage</t>
+  </si>
+  <si>
+    <t>unit</t>
+  </si>
+  <si>
+    <t>instructions</t>
+  </si>
+  <si>
+    <t>Nhóm Hồ sơ bệnh án (Mối quan hệ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MedicalRecord </t>
+  </si>
+  <si>
+    <t>PrescriptionItem</t>
+  </si>
+  <si>
+    <t>MedicalRecordAttachment</t>
+  </si>
+  <si>
+    <t>signed_at</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -291,8 +384,56 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF555555"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="21">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -394,8 +535,24 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="22">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -577,54 +734,29 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="medium">
-        <color indexed="64"/>
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
@@ -637,80 +769,40 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
       </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="10" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -739,9 +831,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -774,53 +863,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="14" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="15" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="16" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="14" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="15" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="16" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -829,9 +873,78 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="4" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="4" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="18" borderId="4" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="4" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="17" borderId="4" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="6">
+    <cellStyle name="20% - Accent1" xfId="4" builtinId="30"/>
     <cellStyle name="60% - Accent5" xfId="2" builtinId="48"/>
+    <cellStyle name="Accent1" xfId="3" builtinId="29"/>
+    <cellStyle name="Accent2" xfId="5" builtinId="33"/>
     <cellStyle name="Accent5" xfId="1" builtinId="45"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -1176,29 +1289,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2"/>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="12" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="2"/>
-      <c r="E1" s="42" t="s">
+      <c r="E1" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="12"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
-      <c r="P1" s="1"/>
-      <c r="Q1" s="1"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="21"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="21"/>
+      <c r="Q1" s="11"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -1210,29 +1316,33 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A2" s="43" t="s">
+      <c r="A2" s="26" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="2"/>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D2" s="2"/>
-      <c r="E2" s="43" t="s">
+      <c r="E2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
-      <c r="P2" s="1"/>
-      <c r="Q2" s="1"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="43" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" s="44"/>
+      <c r="J2" s="44"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="21"/>
+      <c r="M2" s="41" t="s">
+        <v>83</v>
+      </c>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
+      <c r="Q2" s="11"/>
       <c r="R2" s="1"/>
       <c r="S2" s="1"/>
       <c r="T2" s="1"/>
@@ -1244,29 +1354,33 @@
       <c r="Z2" s="1"/>
     </row>
     <row r="3" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A3" s="43" t="s">
+      <c r="A3" s="26" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D3" s="2"/>
-      <c r="E3" s="43" t="s">
+      <c r="E3" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
-      <c r="P3" s="1"/>
-      <c r="Q3" s="1"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="I3" s="37"/>
+      <c r="J3" s="37"/>
+      <c r="K3" s="11"/>
+      <c r="L3" s="21"/>
+      <c r="M3" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="11"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -1278,29 +1392,33 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A4" s="43" t="s">
+      <c r="A4" s="26" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="2"/>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="2"/>
-      <c r="E4" s="43" t="s">
+      <c r="E4" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="12"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
-      <c r="P4" s="1"/>
-      <c r="Q4" s="1"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="37" t="s">
+        <v>68</v>
+      </c>
+      <c r="I4" s="37"/>
+      <c r="J4" s="37"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="N4" s="37"/>
+      <c r="O4" s="37"/>
+      <c r="P4" s="37"/>
+      <c r="Q4" s="11"/>
       <c r="R4" s="1"/>
       <c r="S4" s="1"/>
       <c r="T4" s="1"/>
@@ -1312,29 +1430,33 @@
       <c r="Z4" s="1"/>
     </row>
     <row r="5" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A5" s="43" t="s">
+      <c r="A5" s="26" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="2"/>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2"/>
-      <c r="E5" s="43" t="s">
+      <c r="E5" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
-      <c r="P5" s="1"/>
-      <c r="Q5" s="1"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="I5" s="37"/>
+      <c r="J5" s="37"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="N5" s="37"/>
+      <c r="O5" s="37"/>
+      <c r="P5" s="37"/>
+      <c r="Q5" s="11"/>
       <c r="R5" s="1"/>
       <c r="S5" s="1"/>
       <c r="T5" s="1"/>
@@ -1346,29 +1468,33 @@
       <c r="Z5" s="1"/>
     </row>
     <row r="6" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A6" s="43" t="s">
+      <c r="A6" s="26" t="s">
         <v>12</v>
       </c>
       <c r="B6" s="2"/>
-      <c r="C6" s="11" t="s">
+      <c r="C6" s="10" t="s">
         <v>55</v>
       </c>
       <c r="D6" s="2"/>
-      <c r="E6" s="44" t="s">
+      <c r="E6" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="F6" s="12"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
-      <c r="P6" s="1"/>
-      <c r="Q6" s="1"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="37"/>
+      <c r="J6" s="37"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="21"/>
+      <c r="M6" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" s="37"/>
+      <c r="O6" s="37"/>
+      <c r="P6" s="37"/>
+      <c r="Q6" s="11"/>
       <c r="R6" s="1"/>
       <c r="S6" s="1"/>
       <c r="T6" s="1"/>
@@ -1380,27 +1506,31 @@
       <c r="Z6" s="1"/>
     </row>
     <row r="7" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="26" t="s">
         <v>13</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
-      <c r="E7" s="43" t="s">
+      <c r="E7" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="F7" s="12"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="1"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="I7" s="37"/>
+      <c r="J7" s="37"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="31"/>
+      <c r="M7" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="N7" s="37"/>
+      <c r="O7" s="37"/>
+      <c r="P7" s="37"/>
+      <c r="Q7" s="11"/>
       <c r="R7" s="1"/>
       <c r="S7" s="1"/>
       <c r="T7" s="1"/>
@@ -1412,26 +1542,30 @@
       <c r="Z7" s="1"/>
     </row>
     <row r="8" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A8" s="43" t="s">
+      <c r="A8" s="26" t="s">
         <v>15</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="16" t="s">
+      <c r="C8" s="29" t="s">
         <v>17</v>
       </c>
       <c r="D8" s="2"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
-      <c r="P8" s="1"/>
-      <c r="Q8" s="1"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="21"/>
+      <c r="H8" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="37"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="21"/>
+      <c r="M8" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="N8" s="37"/>
+      <c r="O8" s="37"/>
+      <c r="P8" s="37"/>
+      <c r="Q8" s="11"/>
       <c r="R8" s="1"/>
       <c r="S8" s="1"/>
       <c r="T8" s="1"/>
@@ -1443,26 +1577,28 @@
       <c r="Z8" s="1"/>
     </row>
     <row r="9" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="27" t="s">
         <v>55</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="26" t="s">
         <v>3</v>
       </c>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="37" t="s">
+        <v>72</v>
+      </c>
+      <c r="I9" s="37"/>
+      <c r="J9" s="37"/>
+      <c r="K9" s="11"/>
       <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
+      <c r="M9" s="23"/>
+      <c r="N9" s="23"/>
+      <c r="O9" s="23"/>
+      <c r="P9" s="23"/>
       <c r="Q9" s="1"/>
       <c r="R9" s="1"/>
       <c r="S9" s="1"/>
@@ -1475,23 +1611,27 @@
       <c r="Z9" s="1"/>
     </row>
     <row r="10" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="26" t="s">
         <v>64</v>
       </c>
       <c r="B10" s="2"/>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="26" t="s">
         <v>20</v>
       </c>
       <c r="D10" s="2"/>
-      <c r="E10" s="41"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="3"/>
-      <c r="K10" s="1"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="37" t="s">
+        <v>73</v>
+      </c>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="11"/>
       <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="M10" s="22"/>
+      <c r="N10" s="22"/>
+      <c r="O10" s="22"/>
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
@@ -1505,22 +1645,24 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A11" s="43" t="s">
+      <c r="A11" s="26" t="s">
         <v>11</v>
       </c>
       <c r="B11" s="2"/>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="26" t="s">
         <v>19</v>
       </c>
       <c r="D11" s="2"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="42" t="s">
+        <v>74</v>
+      </c>
+      <c r="I11" s="42"/>
+      <c r="J11" s="42"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="21"/>
+      <c r="P11" s="11"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
       <c r="S11" s="1"/>
@@ -1534,21 +1676,28 @@
     </row>
     <row r="12" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="2"/>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="26" t="s">
         <v>23</v>
       </c>
       <c r="D12" s="2"/>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="42" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" s="42"/>
+      <c r="J12" s="42"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="40" t="s">
+        <v>87</v>
+      </c>
+      <c r="N12" s="40"/>
+      <c r="O12" s="40"/>
+      <c r="P12" s="11"/>
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
       <c r="S12" s="1"/>
@@ -1562,21 +1711,28 @@
     </row>
     <row r="13" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B13" s="2"/>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="26" t="s">
         <v>26</v>
       </c>
       <c r="D13" s="2"/>
-      <c r="E13" s="9" t="s">
+      <c r="E13" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F13" s="12"/>
-      <c r="G13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="42" t="s">
+        <v>76</v>
+      </c>
+      <c r="I13" s="42"/>
+      <c r="J13" s="42"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="N13" s="37"/>
+      <c r="O13" s="37"/>
+      <c r="P13" s="11"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
       <c r="S13" s="1"/>
@@ -1589,25 +1745,32 @@
       <c r="Z13" s="1"/>
     </row>
     <row r="14" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B14" s="2"/>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="26" t="s">
         <v>28</v>
       </c>
       <c r="D14" s="2"/>
-      <c r="E14" s="9" t="s">
+      <c r="E14" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="F14" s="12"/>
-      <c r="G14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="I14" s="42"/>
+      <c r="J14" s="42"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="21"/>
+      <c r="M14" s="37" t="s">
+        <v>88</v>
+      </c>
+      <c r="N14" s="37"/>
+      <c r="O14" s="37"/>
+      <c r="P14" s="11"/>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
       <c r="S14" s="1"/>
@@ -1620,25 +1783,32 @@
       <c r="Z14" s="1"/>
     </row>
     <row r="15" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B15" s="2"/>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="26" t="s">
         <v>21</v>
       </c>
       <c r="D15" s="2"/>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F15" s="12"/>
-      <c r="G15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="42" t="s">
+        <v>78</v>
+      </c>
+      <c r="I15" s="42"/>
+      <c r="J15" s="42"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="37" t="s">
+        <v>89</v>
+      </c>
+      <c r="N15" s="37"/>
+      <c r="O15" s="37"/>
+      <c r="P15" s="11"/>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
       <c r="S15" s="1"/>
@@ -1651,25 +1821,32 @@
       <c r="Z15" s="1"/>
     </row>
     <row r="16" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="8" t="s">
         <v>19</v>
       </c>
       <c r="B16" s="2"/>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="26" t="s">
         <v>22</v>
       </c>
       <c r="D16" s="2"/>
-      <c r="E16" s="9" t="s">
+      <c r="E16" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F16" s="12"/>
-      <c r="G16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
-      <c r="P16" s="1"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="I16" s="42"/>
+      <c r="J16" s="42"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="21"/>
+      <c r="M16" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="N16" s="37"/>
+      <c r="O16" s="37"/>
+      <c r="P16" s="32"/>
       <c r="Q16" s="1"/>
       <c r="R16" s="1"/>
       <c r="S16" s="1"/>
@@ -1682,26 +1859,33 @@
       <c r="Z16" s="1"/>
     </row>
     <row r="17" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="8" t="s">
         <v>21</v>
       </c>
       <c r="B17" s="2"/>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="26" t="s">
         <v>32</v>
       </c>
       <c r="D17" s="2"/>
-      <c r="E17" s="9" t="s">
+      <c r="E17" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="F17" s="12"/>
-      <c r="G17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="42" t="s">
+        <v>80</v>
+      </c>
+      <c r="I17" s="42"/>
+      <c r="J17" s="42"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="N17" s="37"/>
+      <c r="O17" s="37"/>
+      <c r="P17" s="34"/>
+      <c r="Q17" s="11"/>
       <c r="R17" s="1"/>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
@@ -1713,25 +1897,32 @@
       <c r="Z17" s="1"/>
     </row>
     <row r="18" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="8" t="s">
         <v>22</v>
       </c>
       <c r="B18" s="2"/>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="26" t="s">
         <v>34</v>
       </c>
       <c r="D18" s="2"/>
-      <c r="E18" s="9" t="s">
+      <c r="E18" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="12"/>
-      <c r="G18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="42" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="42"/>
+      <c r="J18" s="42"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="21"/>
+      <c r="M18" s="37" t="s">
+        <v>91</v>
+      </c>
+      <c r="N18" s="37"/>
+      <c r="O18" s="37"/>
+      <c r="P18" s="33"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
       <c r="S18" s="1"/>
@@ -1744,25 +1935,32 @@
       <c r="Z18" s="1"/>
     </row>
     <row r="19" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="8" t="s">
         <v>25</v>
       </c>
       <c r="B19" s="2"/>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="26" t="s">
         <v>35</v>
       </c>
       <c r="D19" s="2"/>
-      <c r="E19" s="9" t="s">
+      <c r="E19" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="F19" s="12"/>
-      <c r="G19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="42" t="s">
+        <v>33</v>
+      </c>
+      <c r="I19" s="42"/>
+      <c r="J19" s="42"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="37" t="s">
+        <v>84</v>
+      </c>
+      <c r="N19" s="37"/>
+      <c r="O19" s="37"/>
+      <c r="P19" s="11"/>
       <c r="Q19" s="1"/>
       <c r="R19" s="1"/>
       <c r="S19" s="1"/>
@@ -1775,57 +1973,84 @@
       <c r="Z19" s="1"/>
     </row>
     <row r="20" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="9" t="s">
         <v>36</v>
       </c>
       <c r="B20" s="2"/>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="26" t="s">
         <v>36</v>
       </c>
       <c r="D20" s="2"/>
-      <c r="E20" s="9" t="s">
+      <c r="E20" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F20" s="14"/>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="42" t="s">
+        <v>82</v>
+      </c>
+      <c r="I20" s="42"/>
+      <c r="J20" s="42"/>
+      <c r="K20" s="13"/>
     </row>
     <row r="21" spans="1:26" ht="19" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
-      <c r="C21" s="11" t="s">
+      <c r="C21" s="27" t="s">
         <v>55</v>
       </c>
       <c r="D21" s="2"/>
-      <c r="E21" s="9" t="s">
+      <c r="E21" s="8" t="s">
         <v>33</v>
       </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="42" t="s">
+        <v>67</v>
+      </c>
+      <c r="I21" s="42"/>
+      <c r="J21" s="42"/>
+      <c r="K21" s="13"/>
     </row>
     <row r="22" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A22" s="2"/>
       <c r="B22" s="2"/>
+      <c r="C22" s="26" t="s">
+        <v>62</v>
+      </c>
       <c r="D22" s="2"/>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="10" t="s">
         <v>55</v>
       </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="42" t="s">
+        <v>36</v>
+      </c>
+      <c r="I22" s="42"/>
+      <c r="J22" s="42"/>
+      <c r="K22" s="13"/>
     </row>
     <row r="23" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A23" s="2"/>
       <c r="B23" s="2"/>
-      <c r="C23" s="17" t="s">
+      <c r="C23" s="15" t="s">
         <v>38</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="1"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="14"/>
-      <c r="K23" s="24"/>
-      <c r="L23" s="24"/>
-      <c r="M23" s="24"/>
+      <c r="G23" s="47"/>
+      <c r="H23" s="42" t="s">
+        <v>96</v>
+      </c>
+      <c r="I23" s="42"/>
+      <c r="J23" s="42"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="22"/>
       <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
-      <c r="P23" s="1"/>
-      <c r="Q23" s="1"/>
+      <c r="O23" s="22"/>
+      <c r="P23" s="22"/>
+      <c r="Q23" s="22"/>
       <c r="R23" s="1"/>
       <c r="S23" s="1"/>
       <c r="T23" s="1"/>
@@ -1837,34 +2062,23 @@
       <c r="Z23" s="1"/>
     </row>
     <row r="24" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="20" t="s">
         <v>37</v>
       </c>
       <c r="B24" s="2"/>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D24" s="2"/>
-      <c r="E24" s="18" t="s">
+      <c r="E24" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="F24" s="26"/>
-      <c r="G24" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="H24" s="39"/>
-      <c r="I24" s="40"/>
-      <c r="J24" s="26"/>
-      <c r="K24" s="35" t="s">
-        <v>56</v>
-      </c>
-      <c r="L24" s="36"/>
-      <c r="M24" s="37"/>
-      <c r="N24" s="12"/>
-      <c r="O24" s="1"/>
-      <c r="P24" s="1"/>
-      <c r="Q24" s="1"/>
-      <c r="R24" s="1"/>
+      <c r="F24" s="24"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="48"/>
+      <c r="N24" s="24"/>
+      <c r="R24" s="11"/>
       <c r="S24" s="1"/>
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
@@ -1875,34 +2089,21 @@
       <c r="Z24" s="1"/>
     </row>
     <row r="25" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B25" s="2"/>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D25" s="2"/>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F25" s="26"/>
-      <c r="G25" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="H25" s="28"/>
-      <c r="I25" s="29"/>
-      <c r="J25" s="26"/>
-      <c r="K25" s="27" t="s">
-        <v>3</v>
-      </c>
-      <c r="L25" s="28"/>
-      <c r="M25" s="29"/>
-      <c r="N25" s="12"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
+      <c r="F25" s="24"/>
+      <c r="J25" s="24"/>
+      <c r="N25" s="24"/>
+      <c r="R25" s="11"/>
       <c r="S25" s="1"/>
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
@@ -1913,34 +2114,21 @@
       <c r="Z25" s="1"/>
     </row>
     <row r="26" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="8" t="s">
         <v>40</v>
       </c>
       <c r="B26" s="2"/>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="2"/>
-      <c r="E26" s="9" t="s">
+      <c r="E26" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="F26" s="26"/>
-      <c r="G26" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="H26" s="28"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="27" t="s">
-        <v>20</v>
-      </c>
-      <c r="L26" s="28"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="1"/>
-      <c r="P26" s="1"/>
-      <c r="Q26" s="1"/>
-      <c r="R26" s="1"/>
+      <c r="F26" s="24"/>
+      <c r="J26" s="24"/>
+      <c r="N26" s="24"/>
+      <c r="R26" s="11"/>
       <c r="S26" s="1"/>
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
@@ -1951,34 +2139,21 @@
       <c r="Z26" s="1"/>
     </row>
     <row r="27" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="17" t="s">
         <v>41</v>
       </c>
       <c r="B27" s="2"/>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>29</v>
       </c>
       <c r="D27" s="2"/>
-      <c r="E27" s="19" t="s">
+      <c r="E27" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="F27" s="26"/>
-      <c r="G27" s="27" t="s">
-        <v>23</v>
-      </c>
-      <c r="H27" s="28"/>
-      <c r="I27" s="29"/>
-      <c r="J27" s="26"/>
-      <c r="K27" s="27" t="s">
-        <v>57</v>
-      </c>
-      <c r="L27" s="28"/>
-      <c r="M27" s="29"/>
-      <c r="N27" s="12"/>
-      <c r="O27" s="1"/>
-      <c r="P27" s="1"/>
-      <c r="Q27" s="1"/>
-      <c r="R27" s="1"/>
+      <c r="F27" s="24"/>
+      <c r="J27" s="24"/>
+      <c r="N27" s="24"/>
+      <c r="R27" s="11"/>
       <c r="S27" s="1"/>
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
@@ -1991,28 +2166,15 @@
     <row r="28" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A28" s="2"/>
       <c r="B28" s="2"/>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>14</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
-      <c r="F28" s="23"/>
-      <c r="G28" s="27" t="s">
-        <v>47</v>
-      </c>
-      <c r="H28" s="28"/>
-      <c r="I28" s="29"/>
-      <c r="J28" s="26"/>
-      <c r="K28" s="27" t="s">
-        <v>58</v>
-      </c>
-      <c r="L28" s="28"/>
-      <c r="M28" s="29"/>
-      <c r="N28" s="12"/>
-      <c r="O28" s="1"/>
-      <c r="P28" s="1"/>
-      <c r="Q28" s="1"/>
-      <c r="R28" s="1"/>
+      <c r="F28" s="21"/>
+      <c r="J28" s="24"/>
+      <c r="N28" s="24"/>
+      <c r="R28" s="11"/>
       <c r="S28" s="1"/>
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
@@ -2025,28 +2187,20 @@
     <row r="29" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A29" s="2"/>
       <c r="B29" s="2"/>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>42</v>
       </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
-      <c r="F29" s="23"/>
-      <c r="G29" s="30" t="s">
-        <v>14</v>
+      <c r="F29" s="21"/>
+      <c r="J29" s="24"/>
+      <c r="K29" s="50" t="s">
+        <v>56</v>
       </c>
-      <c r="H29" s="31"/>
-      <c r="I29" s="32"/>
-      <c r="J29" s="26"/>
-      <c r="K29" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L29" s="28"/>
-      <c r="M29" s="29"/>
-      <c r="N29" s="12"/>
-      <c r="O29" s="1"/>
-      <c r="P29" s="1"/>
-      <c r="Q29" s="1"/>
-      <c r="R29" s="1"/>
+      <c r="L29" s="50"/>
+      <c r="M29" s="50"/>
+      <c r="N29" s="24"/>
+      <c r="R29" s="11"/>
       <c r="S29" s="1"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
@@ -2059,28 +2213,27 @@
     <row r="30" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A30" s="2"/>
       <c r="B30" s="2"/>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="9" t="s">
         <v>55</v>
       </c>
       <c r="D30" s="2"/>
-      <c r="E30" s="20" t="s">
+      <c r="E30" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="F30" s="12"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
-      <c r="J30" s="23"/>
-      <c r="K30" s="27" t="s">
-        <v>60</v>
+      <c r="F30" s="24"/>
+      <c r="G30" s="49" t="s">
+        <v>61</v>
       </c>
-      <c r="L30" s="28"/>
-      <c r="M30" s="29"/>
-      <c r="N30" s="12"/>
-      <c r="O30" s="1"/>
-      <c r="P30" s="1"/>
-      <c r="Q30" s="1"/>
-      <c r="R30" s="1"/>
+      <c r="H30" s="49"/>
+      <c r="I30" s="49"/>
+      <c r="J30" s="24"/>
+      <c r="K30" s="37" t="s">
+        <v>3</v>
+      </c>
+      <c r="L30" s="37"/>
+      <c r="M30" s="37"/>
+      <c r="N30" s="24"/>
+      <c r="R30" s="11"/>
       <c r="S30" s="1"/>
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
@@ -2094,24 +2247,23 @@
       <c r="A31" s="2"/>
       <c r="B31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="9" t="s">
+      <c r="E31" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="F31" s="12"/>
-      <c r="G31" s="1"/>
-      <c r="H31" s="1"/>
-      <c r="I31" s="1"/>
-      <c r="J31" s="23"/>
-      <c r="K31" s="27" t="s">
-        <v>33</v>
+      <c r="F31" s="24"/>
+      <c r="G31" s="37" t="s">
+        <v>3</v>
       </c>
-      <c r="L31" s="28"/>
-      <c r="M31" s="29"/>
-      <c r="N31" s="12"/>
-      <c r="O31" s="1"/>
-      <c r="P31" s="1"/>
-      <c r="Q31" s="1"/>
-      <c r="R31" s="1"/>
+      <c r="H31" s="37"/>
+      <c r="I31" s="37"/>
+      <c r="J31" s="24"/>
+      <c r="K31" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="L31" s="37"/>
+      <c r="M31" s="37"/>
+      <c r="N31" s="24"/>
+      <c r="R31" s="11"/>
       <c r="S31" s="1"/>
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
@@ -2122,32 +2274,31 @@
       <c r="Z31" s="1"/>
     </row>
     <row r="32" spans="1:26" ht="25" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A32" s="21" t="s">
+      <c r="A32" s="19" t="s">
         <v>43</v>
       </c>
       <c r="B32" s="2"/>
-      <c r="C32" s="21" t="s">
+      <c r="C32" s="19" t="s">
         <v>44</v>
       </c>
       <c r="D32" s="2"/>
-      <c r="E32" s="9" t="s">
+      <c r="E32" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F32" s="12"/>
-      <c r="G32" s="1"/>
-      <c r="H32" s="1"/>
-      <c r="I32" s="1"/>
-      <c r="J32" s="23"/>
-      <c r="K32" s="30" t="s">
-        <v>55</v>
+      <c r="F32" s="24"/>
+      <c r="G32" s="37" t="s">
+        <v>62</v>
       </c>
-      <c r="L32" s="31"/>
-      <c r="M32" s="32"/>
-      <c r="N32" s="12"/>
-      <c r="O32" s="1"/>
-      <c r="P32" s="1"/>
-      <c r="Q32" s="1"/>
-      <c r="R32" s="1"/>
+      <c r="H32" s="37"/>
+      <c r="I32" s="37"/>
+      <c r="J32" s="24"/>
+      <c r="K32" s="37" t="s">
+        <v>57</v>
+      </c>
+      <c r="L32" s="37"/>
+      <c r="M32" s="37"/>
+      <c r="N32" s="24"/>
+      <c r="R32" s="11"/>
       <c r="S32" s="1"/>
       <c r="T32" s="1"/>
       <c r="U32" s="1"/>
@@ -2158,30 +2309,34 @@
       <c r="Z32" s="1"/>
     </row>
     <row r="33" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="8" t="s">
         <v>3</v>
       </c>
       <c r="B33" s="2"/>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>3</v>
       </c>
       <c r="D33" s="2"/>
-      <c r="E33" s="9" t="s">
+      <c r="E33" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F33" s="12"/>
-      <c r="G33" s="1"/>
-      <c r="H33" s="1"/>
-      <c r="I33" s="1"/>
-      <c r="J33" s="1"/>
-      <c r="K33" s="25"/>
-      <c r="L33" s="25"/>
-      <c r="M33" s="25"/>
-      <c r="N33" s="1"/>
-      <c r="O33" s="1"/>
-      <c r="P33" s="1"/>
-      <c r="Q33" s="1"/>
-      <c r="R33" s="1"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="37" t="s">
+        <v>23</v>
+      </c>
+      <c r="H33" s="37"/>
+      <c r="I33" s="37"/>
+      <c r="J33" s="24"/>
+      <c r="K33" s="37" t="s">
+        <v>58</v>
+      </c>
+      <c r="L33" s="37"/>
+      <c r="M33" s="37"/>
+      <c r="N33" s="24"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="11"/>
       <c r="S33" s="1"/>
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
@@ -2192,30 +2347,34 @@
       <c r="Z33" s="1"/>
     </row>
     <row r="34" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="8" t="s">
         <v>20</v>
       </c>
       <c r="B34" s="2"/>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>46</v>
       </c>
       <c r="D34" s="2"/>
-      <c r="E34" s="9" t="s">
+      <c r="E34" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F34" s="12"/>
-      <c r="G34" s="1"/>
-      <c r="H34" s="1"/>
-      <c r="I34" s="1"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="1"/>
-      <c r="M34" s="1"/>
-      <c r="N34" s="1"/>
-      <c r="O34" s="1"/>
-      <c r="P34" s="1"/>
-      <c r="Q34" s="1"/>
-      <c r="R34" s="1"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="37" t="s">
+        <v>47</v>
+      </c>
+      <c r="H34" s="37"/>
+      <c r="I34" s="37"/>
+      <c r="J34" s="24"/>
+      <c r="K34" s="37" t="s">
+        <v>59</v>
+      </c>
+      <c r="L34" s="37"/>
+      <c r="M34" s="37"/>
+      <c r="N34" s="24"/>
+      <c r="O34" s="46"/>
+      <c r="P34" s="46"/>
+      <c r="Q34" s="46"/>
+      <c r="R34" s="11"/>
       <c r="S34" s="1"/>
       <c r="T34" s="1"/>
       <c r="U34" s="1"/>
@@ -2226,30 +2385,34 @@
       <c r="Z34" s="1"/>
     </row>
     <row r="35" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A35" s="19" t="s">
+      <c r="A35" s="17" t="s">
         <v>36</v>
       </c>
       <c r="B35" s="2"/>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>23</v>
       </c>
       <c r="D35" s="2"/>
-      <c r="E35" s="9" t="s">
+      <c r="E35" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="F35" s="12"/>
-      <c r="G35" s="1"/>
-      <c r="H35" s="1"/>
-      <c r="I35" s="1"/>
-      <c r="J35" s="1"/>
-      <c r="K35" s="1"/>
-      <c r="L35" s="1"/>
-      <c r="M35" s="1"/>
-      <c r="N35" s="1"/>
-      <c r="O35" s="1"/>
-      <c r="P35" s="1"/>
-      <c r="Q35" s="1"/>
-      <c r="R35" s="1"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H35" s="37"/>
+      <c r="I35" s="37"/>
+      <c r="J35" s="24"/>
+      <c r="K35" s="37" t="s">
+        <v>60</v>
+      </c>
+      <c r="L35" s="37"/>
+      <c r="M35" s="37"/>
+      <c r="N35" s="24"/>
+      <c r="O35" s="46"/>
+      <c r="P35" s="46"/>
+      <c r="Q35" s="46"/>
+      <c r="R35" s="11"/>
       <c r="S35" s="1"/>
       <c r="T35" s="1"/>
       <c r="U35" s="1"/>
@@ -2262,26 +2425,28 @@
     <row r="36" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A36" s="2"/>
       <c r="B36" s="2"/>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>47</v>
       </c>
       <c r="D36" s="2"/>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="F36" s="12"/>
-      <c r="G36" s="1"/>
-      <c r="H36" s="1"/>
-      <c r="I36" s="1"/>
-      <c r="J36" s="1"/>
-      <c r="K36" s="1"/>
-      <c r="L36" s="1"/>
-      <c r="M36" s="1"/>
-      <c r="N36" s="1"/>
-      <c r="O36" s="1"/>
-      <c r="P36" s="1"/>
-      <c r="Q36" s="1"/>
-      <c r="R36" s="1"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="46"/>
+      <c r="H36" s="46"/>
+      <c r="I36" s="46"/>
+      <c r="J36" s="24"/>
+      <c r="K36" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="L36" s="37"/>
+      <c r="M36" s="37"/>
+      <c r="N36" s="24"/>
+      <c r="O36" s="46"/>
+      <c r="P36" s="46"/>
+      <c r="Q36" s="46"/>
+      <c r="R36" s="11"/>
       <c r="S36" s="1"/>
       <c r="T36" s="1"/>
       <c r="U36" s="1"/>
@@ -2294,22 +2459,24 @@
     <row r="37" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A37" s="2"/>
       <c r="B37" s="2"/>
-      <c r="C37" s="19" t="s">
+      <c r="C37" s="17" t="s">
         <v>14</v>
       </c>
       <c r="D37" s="2"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="J37" s="1"/>
-      <c r="K37" s="1"/>
-      <c r="L37" s="1"/>
-      <c r="M37" s="1"/>
-      <c r="N37" s="1"/>
-      <c r="O37" s="1"/>
-      <c r="P37" s="1"/>
-      <c r="Q37" s="1"/>
+      <c r="G37" s="23"/>
+      <c r="H37" s="23"/>
+      <c r="I37" s="23"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="L37" s="37"/>
+      <c r="M37" s="37"/>
+      <c r="N37" s="11"/>
+      <c r="O37" s="23"/>
+      <c r="P37" s="23"/>
+      <c r="Q37" s="23"/>
       <c r="R37" s="1"/>
       <c r="S37" s="1"/>
       <c r="T37" s="1"/>
@@ -2329,11 +2496,11 @@
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
       <c r="I38" s="1"/>
-      <c r="J38" s="1"/>
-      <c r="K38" s="1"/>
-      <c r="L38" s="1"/>
-      <c r="M38" s="1"/>
-      <c r="N38" s="1"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="11"/>
       <c r="O38" s="1"/>
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
@@ -2348,22 +2515,22 @@
       <c r="Z38" s="1"/>
     </row>
     <row r="39" spans="1:26" ht="26.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="33" t="s">
+      <c r="A39" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="B39" s="34"/>
-      <c r="C39" s="34"/>
-      <c r="D39" s="34"/>
-      <c r="E39" s="34"/>
+      <c r="B39" s="39"/>
+      <c r="C39" s="39"/>
+      <c r="D39" s="39"/>
+      <c r="E39" s="39"/>
       <c r="F39" s="1"/>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
-      <c r="J39" s="1"/>
-      <c r="K39" s="1"/>
-      <c r="L39" s="1"/>
-      <c r="M39" s="1"/>
-      <c r="N39" s="1"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="46"/>
+      <c r="L39" s="46"/>
+      <c r="M39" s="46"/>
+      <c r="N39" s="11"/>
       <c r="O39" s="1"/>
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
@@ -2378,13 +2545,13 @@
       <c r="Z39" s="1"/>
     </row>
     <row r="40" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A40" s="4">
+      <c r="A40" s="3">
         <v>1</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="C40" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D40" s="2"/>
@@ -2393,11 +2560,11 @@
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
-      <c r="J40" s="1"/>
-      <c r="K40" s="1"/>
-      <c r="L40" s="1"/>
-      <c r="M40" s="1"/>
-      <c r="N40" s="1"/>
+      <c r="J40" s="21"/>
+      <c r="K40" s="46"/>
+      <c r="L40" s="46"/>
+      <c r="M40" s="46"/>
+      <c r="N40" s="11"/>
       <c r="O40" s="1"/>
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
@@ -2412,13 +2579,13 @@
       <c r="Z40" s="1"/>
     </row>
     <row r="41" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B41" s="7" t="s">
+      <c r="B41" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C41" s="6" t="s">
+      <c r="C41" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D41" s="2"/>
@@ -2428,9 +2595,9 @@
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
-      <c r="K41" s="1"/>
-      <c r="L41" s="1"/>
-      <c r="M41" s="1"/>
+      <c r="K41" s="23"/>
+      <c r="L41" s="23"/>
+      <c r="M41" s="23"/>
       <c r="N41" s="1"/>
       <c r="O41" s="1"/>
       <c r="P41" s="1"/>
@@ -2474,13 +2641,13 @@
       <c r="Z42" s="1"/>
     </row>
     <row r="43" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A43" s="4">
+      <c r="A43" s="3">
         <v>1</v>
       </c>
-      <c r="B43" s="5" t="s">
+      <c r="B43" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C43" s="4" t="s">
+      <c r="C43" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D43" s="2"/>
@@ -2508,13 +2675,13 @@
       <c r="Z43" s="1"/>
     </row>
     <row r="44" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A44" s="6" t="s">
+      <c r="A44" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B44" s="7" t="s">
+      <c r="B44" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="5" t="s">
         <v>2</v>
       </c>
       <c r="D44" s="2"/>
@@ -2570,13 +2737,13 @@
       <c r="Z45" s="1"/>
     </row>
     <row r="46" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A46" s="4">
+      <c r="A46" s="3">
         <v>1</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C46" s="4" t="s">
+      <c r="C46" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D46" s="2"/>
@@ -2604,13 +2771,13 @@
       <c r="Z46" s="1"/>
     </row>
     <row r="47" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A47" s="6" t="s">
+      <c r="A47" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B47" s="7" t="s">
+      <c r="B47" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="5" t="s">
         <v>16</v>
       </c>
       <c r="D47" s="2"/>
@@ -2666,13 +2833,13 @@
       <c r="Z48" s="1"/>
     </row>
     <row r="49" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A49" s="4">
+      <c r="A49" s="3">
         <v>1</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C49" s="4" t="s">
+      <c r="C49" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D49" s="2"/>
@@ -2700,13 +2867,13 @@
       <c r="Z49" s="1"/>
     </row>
     <row r="50" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B50" s="7" t="s">
+      <c r="B50" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D50" s="2"/>
@@ -2762,13 +2929,13 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A52" s="4">
+      <c r="A52" s="3">
         <v>1</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C52" s="4" t="s">
+      <c r="C52" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D52" s="2"/>
@@ -2796,13 +2963,13 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B53" s="7" t="s">
+      <c r="B53" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C53" s="6" t="s">
+      <c r="C53" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D53" s="2"/>
@@ -2858,13 +3025,13 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A55" s="4">
+      <c r="A55" s="3">
         <v>1</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C55" s="4" t="s">
+      <c r="C55" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D55" s="2"/>
@@ -2892,13 +3059,13 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A56" s="6" t="s">
+      <c r="A56" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B56" s="7" t="s">
+      <c r="B56" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C56" s="6" t="s">
+      <c r="C56" s="5" t="s">
         <v>18</v>
       </c>
       <c r="D56" s="2"/>
@@ -2954,13 +3121,13 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A58" s="4">
+      <c r="A58" s="3">
         <v>1</v>
       </c>
-      <c r="B58" s="5" t="s">
+      <c r="B58" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C58" s="4">
+      <c r="C58" s="3">
         <v>1</v>
       </c>
       <c r="D58" s="2"/>
@@ -2988,13 +3155,13 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A59" s="6" t="s">
+      <c r="A59" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B59" s="7" t="s">
+      <c r="B59" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C59" s="6" t="s">
+      <c r="C59" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D59" s="2"/>
@@ -3022,26 +3189,26 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A60" s="4">
+      <c r="A60" s="3">
         <v>1</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C60" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
     </row>
     <row r="61" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A61" s="6" t="s">
+      <c r="A61" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B61" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C61" s="6" t="s">
+      <c r="C61" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D61" s="2"/>
@@ -3083,13 +3250,13 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" spans="1:26" ht="26.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A64" s="33" t="s">
+      <c r="A64" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B64" s="34"/>
-      <c r="C64" s="34"/>
-      <c r="D64" s="34"/>
-      <c r="E64" s="34"/>
+      <c r="B64" s="39"/>
+      <c r="C64" s="39"/>
+      <c r="D64" s="39"/>
+      <c r="E64" s="39"/>
       <c r="F64" s="1"/>
       <c r="G64" s="1"/>
       <c r="H64" s="1"/>
@@ -3113,13 +3280,13 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A65" s="4">
+      <c r="A65" s="3">
         <v>1</v>
       </c>
-      <c r="B65" s="5" t="s">
+      <c r="B65" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C65" s="4">
+      <c r="C65" s="3">
         <v>1</v>
       </c>
       <c r="D65" s="2"/>
@@ -3147,13 +3314,13 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A66" s="6" t="s">
+      <c r="A66" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="B66" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C66" s="6" t="s">
+      <c r="C66" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D66" s="2"/>
@@ -3209,13 +3376,13 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A68" s="4">
+      <c r="A68" s="3">
         <v>1</v>
       </c>
-      <c r="B68" s="5" t="s">
+      <c r="B68" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C68" s="4" t="s">
+      <c r="C68" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D68" s="2"/>
@@ -3243,13 +3410,13 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A69" s="6" t="s">
+      <c r="A69" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B69" s="7" t="s">
+      <c r="B69" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C69" s="6" t="s">
+      <c r="C69" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D69" s="2"/>
@@ -3305,13 +3472,13 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A71" s="4">
+      <c r="A71" s="3">
         <v>1</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C71" s="4" t="s">
+      <c r="C71" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D71" s="2"/>
@@ -3339,13 +3506,13 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A72" s="6" t="s">
+      <c r="A72" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B72" s="7" t="s">
+      <c r="B72" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C72" s="6" t="s">
+      <c r="C72" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D72" s="2"/>
@@ -3401,13 +3568,13 @@
       <c r="Z73" s="1"/>
     </row>
     <row r="74" spans="1:26" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A74" s="4">
+      <c r="A74" s="3">
         <v>1</v>
       </c>
-      <c r="B74" s="5" t="s">
+      <c r="B74" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C74" s="4">
+      <c r="C74" s="3">
         <v>1</v>
       </c>
       <c r="D74" s="2"/>
@@ -3435,13 +3602,13 @@
       <c r="Z74" s="1"/>
     </row>
     <row r="75" spans="1:26" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A75" s="6" t="s">
+      <c r="A75" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B75" s="7" t="s">
+      <c r="B75" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C75" s="6" t="s">
+      <c r="C75" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D75" s="2"/>
@@ -3497,13 +3664,13 @@
       <c r="Z76" s="1"/>
     </row>
     <row r="77" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A77" s="33" t="s">
+      <c r="A77" s="45" t="s">
         <v>54</v>
       </c>
-      <c r="B77" s="34"/>
-      <c r="C77" s="34"/>
-      <c r="D77" s="34"/>
-      <c r="E77" s="34"/>
+      <c r="B77" s="39"/>
+      <c r="C77" s="39"/>
+      <c r="D77" s="39"/>
+      <c r="E77" s="39"/>
       <c r="F77" s="1"/>
       <c r="G77" s="1"/>
       <c r="H77" s="1"/>
@@ -3527,13 +3694,13 @@
       <c r="Z77" s="1"/>
     </row>
     <row r="78" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A78" s="4">
+      <c r="A78" s="3">
         <v>1</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C78" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D78" s="2"/>
@@ -3561,13 +3728,13 @@
       <c r="Z78" s="1"/>
     </row>
     <row r="79" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A79" s="6" t="s">
+      <c r="A79" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B79" s="7" t="s">
+      <c r="B79" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C79" s="6" t="s">
+      <c r="C79" s="5" t="s">
         <v>63</v>
       </c>
       <c r="D79" s="2"/>
@@ -3623,13 +3790,13 @@
       <c r="Z80" s="1"/>
     </row>
     <row r="81" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A81" s="4">
+      <c r="A81" s="3">
         <v>1</v>
       </c>
-      <c r="B81" s="5" t="s">
+      <c r="B81" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C81" s="4" t="s">
+      <c r="C81" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D81" s="2"/>
@@ -3657,13 +3824,13 @@
       <c r="Z81" s="1"/>
     </row>
     <row r="82" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A82" s="6" t="s">
+      <c r="A82" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B82" s="7" t="s">
+      <c r="B82" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C82" s="6" t="s">
+      <c r="C82" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D82" s="2"/>
@@ -3719,13 +3886,13 @@
       <c r="Z83" s="1"/>
     </row>
     <row r="84" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A84" s="4">
+      <c r="A84" s="3">
         <v>1</v>
       </c>
-      <c r="B84" s="5" t="s">
+      <c r="B84" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C84" s="4" t="s">
+      <c r="C84" s="3" t="s">
         <v>53</v>
       </c>
       <c r="D84" s="2"/>
@@ -3753,13 +3920,13 @@
       <c r="Z84" s="1"/>
     </row>
     <row r="85" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A85" s="6" t="s">
+      <c r="A85" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="B85" s="7" t="s">
+      <c r="B85" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C85" s="6" t="s">
+      <c r="C85" s="5" t="s">
         <v>61</v>
       </c>
       <c r="D85" s="2"/>
@@ -3815,14 +3982,14 @@
       <c r="Z86" s="1"/>
     </row>
     <row r="87" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A87" s="4">
+      <c r="A87" s="3">
         <v>1</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C87" s="4">
-        <v>1</v>
+      <c r="C87" s="35" t="s">
+        <v>53</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="2"/>
@@ -3849,13 +4016,13 @@
       <c r="Z87" s="1"/>
     </row>
     <row r="88" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A88" s="6" t="s">
+      <c r="A88" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="B88" s="7" t="s">
+      <c r="B88" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="5" t="s">
         <v>17</v>
       </c>
       <c r="D88" s="2"/>
@@ -3910,12 +4077,14 @@
       <c r="Y89" s="1"/>
       <c r="Z89" s="1"/>
     </row>
-    <row r="90" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A90" s="2"/>
-      <c r="B90" s="2"/>
-      <c r="C90" s="2"/>
-      <c r="D90" s="2"/>
-      <c r="E90" s="2"/>
+    <row r="90" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A90" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="B90" s="39"/>
+      <c r="C90" s="39"/>
+      <c r="D90" s="39"/>
+      <c r="E90" s="39"/>
       <c r="F90" s="1"/>
       <c r="G90" s="1"/>
       <c r="H90" s="1"/>
@@ -3939,9 +4108,15 @@
       <c r="Z90" s="1"/>
     </row>
     <row r="91" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A91" s="2"/>
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
+      <c r="A91" s="3">
+        <v>1</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C91" s="3">
+        <v>1</v>
+      </c>
       <c r="D91" s="2"/>
       <c r="E91" s="2"/>
       <c r="F91" s="1"/>
@@ -3967,9 +4142,15 @@
       <c r="Z91" s="1"/>
     </row>
     <row r="92" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A92" s="2"/>
-      <c r="B92" s="2"/>
-      <c r="C92" s="2"/>
+      <c r="A92" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C92" s="36" t="s">
+        <v>17</v>
+      </c>
       <c r="D92" s="2"/>
       <c r="E92" s="2"/>
       <c r="F92" s="1"/>
@@ -4023,9 +4204,15 @@
       <c r="Z93" s="1"/>
     </row>
     <row r="94" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A94" s="2"/>
-      <c r="B94" s="2"/>
-      <c r="C94" s="2"/>
+      <c r="A94" s="3">
+        <v>1</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="D94" s="2"/>
       <c r="E94" s="2"/>
       <c r="F94" s="1"/>
@@ -4051,9 +4238,15 @@
       <c r="Z94" s="1"/>
     </row>
     <row r="95" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A95" s="2"/>
-      <c r="B95" s="2"/>
-      <c r="C95" s="2"/>
+      <c r="A95" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C95" s="36" t="s">
+        <v>94</v>
+      </c>
       <c r="D95" s="2"/>
       <c r="E95" s="2"/>
       <c r="F95" s="1"/>
@@ -4107,9 +4300,15 @@
       <c r="Z96" s="1"/>
     </row>
     <row r="97" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A97" s="2"/>
-      <c r="B97" s="2"/>
-      <c r="C97" s="2"/>
+      <c r="A97" s="3">
+        <v>1</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>53</v>
+      </c>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
       <c r="F97" s="1"/>
@@ -4135,9 +4334,15 @@
       <c r="Z97" s="1"/>
     </row>
     <row r="98" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="A98" s="2"/>
-      <c r="B98" s="2"/>
-      <c r="C98" s="2"/>
+      <c r="A98" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C98" s="36" t="s">
+        <v>95</v>
+      </c>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
       <c r="F98" s="1"/>
@@ -4190,12 +4395,12 @@
       <c r="Y99" s="1"/>
       <c r="Z99" s="1"/>
     </row>
-    <row r="100" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A100" s="1"/>
-      <c r="B100" s="1"/>
-      <c r="C100" s="1"/>
-      <c r="D100" s="1"/>
-      <c r="E100" s="1"/>
+    <row r="100" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A100" s="3"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="35"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
       <c r="F100" s="1"/>
       <c r="G100" s="1"/>
       <c r="H100" s="1"/>
@@ -4218,12 +4423,12 @@
       <c r="Y100" s="1"/>
       <c r="Z100" s="1"/>
     </row>
-    <row r="101" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A101" s="1"/>
-      <c r="B101" s="1"/>
-      <c r="C101" s="1"/>
-      <c r="D101" s="1"/>
-      <c r="E101" s="1"/>
+    <row r="101" spans="1:26" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A101" s="5"/>
+      <c r="B101" s="6"/>
+      <c r="C101" s="36"/>
+      <c r="D101" s="2"/>
+      <c r="E101" s="2"/>
       <c r="F101" s="1"/>
       <c r="G101" s="1"/>
       <c r="H101" s="1"/>
@@ -29587,25 +29792,63 @@
       <c r="Z1006" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
+  <mergeCells count="56">
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="A64:E64"/>
     <mergeCell ref="A77:E77"/>
-    <mergeCell ref="K24:M24"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="K27:M27"/>
-    <mergeCell ref="K28:M28"/>
     <mergeCell ref="K29:M29"/>
     <mergeCell ref="K30:M30"/>
     <mergeCell ref="K31:M31"/>
     <mergeCell ref="K32:M32"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
-    <mergeCell ref="G27:I27"/>
-    <mergeCell ref="G28:I28"/>
-    <mergeCell ref="G29:I29"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A64:E64"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="G30:I30"/>
+    <mergeCell ref="G31:I31"/>
+    <mergeCell ref="G32:I32"/>
+    <mergeCell ref="G33:I33"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="H2:J2"/>
+    <mergeCell ref="H3:J3"/>
+    <mergeCell ref="H21:J21"/>
+    <mergeCell ref="H20:J20"/>
+    <mergeCell ref="H19:J19"/>
+    <mergeCell ref="H18:J18"/>
+    <mergeCell ref="H17:J17"/>
+    <mergeCell ref="H16:J16"/>
+    <mergeCell ref="H15:J15"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="H13:J13"/>
+    <mergeCell ref="H22:J22"/>
+    <mergeCell ref="H23:J23"/>
+    <mergeCell ref="M2:P2"/>
+    <mergeCell ref="M4:P4"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="H6:J6"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="M7:P7"/>
+    <mergeCell ref="M6:P6"/>
+    <mergeCell ref="M5:P5"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="A90:E90"/>
+    <mergeCell ref="M13:O13"/>
+    <mergeCell ref="M12:O12"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="M8:P8"/>
+    <mergeCell ref="M18:O18"/>
+    <mergeCell ref="M17:O17"/>
+    <mergeCell ref="M16:O16"/>
+    <mergeCell ref="M15:O15"/>
+    <mergeCell ref="M14:O14"/>
+    <mergeCell ref="H12:J12"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="H8:J8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>